<commit_message>
Agregue la rama original y principal del proyecto
</commit_message>
<xml_diff>
--- a/xls_temporal.xlsx
+++ b/xls_temporal.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,126 +448,126 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>858000029284325</t>
+          <t>858000046476752</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>108</t>
+          <t>27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>858000033124042</t>
+          <t>858000046537810</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>858000034116423</t>
+          <t>858000046629495</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>100</t>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>858000034666725</t>
+          <t>858000050710468</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>97</t>
+          <t>35</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>858000038835778</t>
+          <t>858000050897835</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>858000042728959</t>
+          <t>858000051098300</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>858000043488139</t>
+          <t>858000051107748</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>858000058611410</t>
+          <t>858000051168600</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -577,31 +577,31 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>127</t>
+          <t>36</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>858000058611411</t>
+          <t>858000053573152</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>28</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>858000058611414</t>
+          <t>858000053748915</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -611,14 +611,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>87</t>
+          <t>34</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>858000059403000</t>
+          <t>858000054167253</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -628,31 +628,31 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>858000059403001</t>
+          <t>858000054860373</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>858000059403002</t>
+          <t>858000054860378</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -662,31 +662,31 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>858000059403099</t>
+          <t>858000055115112</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>33</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>858000059403100</t>
+          <t>858000055115117</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -696,14 +696,14 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>33</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>858000059403101</t>
+          <t>858000055679809</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -713,14 +713,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>858000059403102</t>
+          <t>858000055853717</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -730,14 +730,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>26</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>858000059403103</t>
+          <t>858000055853778</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -747,14 +747,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>26</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>858000059403104</t>
+          <t>858000056049621</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -764,48 +764,48 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>25</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>858000059403105</t>
+          <t>858000056066434</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>27</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>858000059403106</t>
+          <t>858000056066436</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>24</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>858000059403107</t>
+          <t>858000056254053</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -815,31 +815,31 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>858000059403108</t>
+          <t>858000056254054</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>858000059403110</t>
+          <t>858000056254126</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -849,14 +849,14 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>858000059403111</t>
+          <t>858000056254137</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -866,31 +866,31 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>29</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>858000059403112</t>
+          <t>858000056334628</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>30</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>858000059403113</t>
+          <t>858000056484849</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -900,48 +900,48 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>31</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>858000059403114</t>
+          <t>858000056554450</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>858000059403115</t>
+          <t>858000056956690</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>858000059403116</t>
+          <t>858000056956694</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -951,14 +951,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>858000059403117</t>
+          <t>858000056956696</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -968,14 +968,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>20</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>858000059403119</t>
+          <t>858000057323204</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -985,31 +985,31 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>13</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>858000059403160</t>
+          <t>858000057376411</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>858000059403161</t>
+          <t>858000057376432</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1019,48 +1019,48 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>858000059403162</t>
+          <t>858000057392460</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>858000059403163</t>
+          <t>858000057393020</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>22</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>858000059403164</t>
+          <t>858000057393057</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1070,14 +1070,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>22</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>858000059403165</t>
+          <t>858000057393125</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1087,14 +1087,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>22</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>858000059403166</t>
+          <t>858000057554205</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1104,14 +1104,14 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>19</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>858000059403167</t>
+          <t>858000057554215</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1121,14 +1121,14 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>19</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>858000059403168</t>
+          <t>858000057832799</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1138,48 +1138,48 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>43</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>858000059403169</t>
+          <t>858000058257967</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>858000059403170</t>
+          <t>858000058257970</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>858000059403171</t>
+          <t>858000058257971</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1189,14 +1189,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>858000059403172</t>
+          <t>858000058257995</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1206,65 +1206,65 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>21</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>858000059403173</t>
+          <t>858000058974492</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>14</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>858000059403174</t>
+          <t>858000059636100</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>858000059403175</t>
+          <t>858000059636104</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>858000059403176</t>
+          <t>858000059636109</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1274,31 +1274,31 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>12</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>858000059403177</t>
+          <t>858000060495141</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>32</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>858000059403178</t>
+          <t>858000061433837</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1308,24 +1308,41 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>858000059403179</t>
+          <t>858000061433838</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>M</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>858000061433839</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>6</t>
         </is>
       </c>
     </row>

</xml_diff>